<commit_message>
Set daynite to import export processes
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/vt_EST_PRI_v1.xlsx
+++ b/VerveStacks_EST/vt_EST_PRI_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AA3FEDE-457E-4A17-AA94-938421A69D38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A72A4B7A-EE69-4D49-9045-CFA0C1907343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="37">
   <si>
     <t>~FI_Process</t>
   </si>
@@ -145,6 +145,9 @@
   </si>
   <si>
     <t>ncap_af</t>
+  </si>
+  <si>
+    <t>daynite</t>
   </si>
 </sst>
 </file>
@@ -596,7 +599,7 @@
         <v>9</v>
       </c>
       <c r="F5" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="H5" t="s">
         <v>30</v>
@@ -646,7 +649,7 @@
         <v>9</v>
       </c>
       <c r="F6" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="H6" t="s">
         <v>30</v>
@@ -693,7 +696,7 @@
         <v>9</v>
       </c>
       <c r="F7" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="H7" t="s">
         <v>30</v>
@@ -713,7 +716,7 @@
         <v>9</v>
       </c>
       <c r="F8" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>